<commit_message>
update website and slide till df
</commit_message>
<xml_diff>
--- a/materials/2_struttureDati/data/df_age.xlsx
+++ b/materials/2_struttureDati/data/df_age.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -365,6 +365,11 @@
           <t>age</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -375,6 +380,11 @@
       <c r="B2">
         <v>20</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -383,7 +393,12 @@
         </is>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>18</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>